<commit_message>
Add data for 2026-10-04
</commit_message>
<xml_diff>
--- a/output/index-crime-full-year.xlsx
+++ b/output/index-crime-full-year.xlsx
@@ -913,7 +913,7 @@
         <v>6588</v>
       </c>
       <c r="M2">
-        <v>4878</v>
+        <v>4895</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -954,7 +954,7 @@
         <v>7126</v>
       </c>
       <c r="M3">
-        <v>5484</v>
+        <v>5506</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1036,7 +1036,7 @@
         <v>6213</v>
       </c>
       <c r="M5">
-        <v>4297</v>
+        <v>4319</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -1077,7 +1077,7 @@
         <v>1956</v>
       </c>
       <c r="M6">
-        <v>1486</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -1118,7 +1118,7 @@
         <v>435</v>
       </c>
       <c r="M7">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -1159,7 +1159,7 @@
         <v>17259</v>
       </c>
       <c r="M8">
-        <v>13826</v>
+        <v>13869</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1200,7 +1200,7 @@
         <v>5816</v>
       </c>
       <c r="M9">
-        <v>3596</v>
+        <v>3615</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1241,7 +1241,7 @@
         <v>58729</v>
       </c>
       <c r="M10">
-        <v>44290</v>
+        <v>44463</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1282,7 +1282,7 @@
         <v>104496</v>
       </c>
       <c r="M11">
-        <v>78476</v>
+        <v>78780</v>
       </c>
     </row>
   </sheetData>
@@ -1389,7 +1389,7 @@
         <v>319</v>
       </c>
       <c r="M2">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -1430,7 +1430,7 @@
         <v>446</v>
       </c>
       <c r="M3">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -1635,7 +1635,7 @@
         <v>636</v>
       </c>
       <c r="M8">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -1676,7 +1676,7 @@
         <v>226</v>
       </c>
       <c r="M9">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1717,7 +1717,7 @@
         <v>1355</v>
       </c>
       <c r="M10">
-        <v>1065</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1758,7 +1758,7 @@
         <v>3388</v>
       </c>
       <c r="M11">
-        <v>2693</v>
+        <v>2702</v>
       </c>
     </row>
   </sheetData>
@@ -2479,7 +2479,7 @@
         <v>221</v>
       </c>
       <c r="M8">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2520,7 +2520,7 @@
         <v>77</v>
       </c>
       <c r="M9">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2561,7 +2561,7 @@
         <v>1200</v>
       </c>
       <c r="M10">
-        <v>999</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2602,7 +2602,7 @@
         <v>1749</v>
       </c>
       <c r="M11">
-        <v>1426</v>
+        <v>1439</v>
       </c>
     </row>
   </sheetData>
@@ -2832,7 +2832,7 @@
         <v>62</v>
       </c>
       <c r="M5">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2952,7 +2952,7 @@
         <v>121</v>
       </c>
       <c r="M8">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3034,7 +3034,7 @@
         <v>819</v>
       </c>
       <c r="M10">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3075,7 +3075,7 @@
         <v>1149</v>
       </c>
       <c r="M11">
-        <v>903</v>
+        <v>906</v>
       </c>
     </row>
   </sheetData>
@@ -3504,7 +3504,7 @@
         <v>321</v>
       </c>
       <c r="M10">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -3545,7 +3545,7 @@
         <v>782</v>
       </c>
       <c r="M11">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
   </sheetData>
@@ -3652,7 +3652,7 @@
         <v>84</v>
       </c>
       <c r="M2">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -3816,7 +3816,7 @@
         <v>12</v>
       </c>
       <c r="M6">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -3898,7 +3898,7 @@
         <v>138</v>
       </c>
       <c r="M8">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -3980,7 +3980,7 @@
         <v>602</v>
       </c>
       <c r="M10">
-        <v>633</v>
+        <v>634</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4021,7 +4021,7 @@
         <v>1011</v>
       </c>
       <c r="M11">
-        <v>932</v>
+        <v>936</v>
       </c>
     </row>
   </sheetData>
@@ -4128,7 +4128,7 @@
         <v>436</v>
       </c>
       <c r="M2">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -4169,7 +4169,7 @@
         <v>503</v>
       </c>
       <c r="M3">
-        <v>374</v>
+        <v>379</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4292,7 +4292,7 @@
         <v>104</v>
       </c>
       <c r="M6">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -4374,7 +4374,7 @@
         <v>778</v>
       </c>
       <c r="M8">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -4415,7 +4415,7 @@
         <v>340</v>
       </c>
       <c r="M9">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -4456,7 +4456,7 @@
         <v>1964</v>
       </c>
       <c r="M10">
-        <v>1390</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4497,7 +4497,7 @@
         <v>4416</v>
       </c>
       <c r="M11">
-        <v>3317</v>
+        <v>3333</v>
       </c>
     </row>
   </sheetData>
@@ -4645,7 +4645,7 @@
         <v>219</v>
       </c>
       <c r="M3">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -4727,7 +4727,7 @@
         <v>194</v>
       </c>
       <c r="M5">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -4932,7 +4932,7 @@
         <v>938</v>
       </c>
       <c r="M10">
-        <v>783</v>
+        <v>786</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -4973,7 +4973,7 @@
         <v>2405</v>
       </c>
       <c r="M11">
-        <v>1737</v>
+        <v>1743</v>
       </c>
     </row>
   </sheetData>
@@ -5080,7 +5080,7 @@
         <v>113</v>
       </c>
       <c r="M2">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -5121,7 +5121,7 @@
         <v>150</v>
       </c>
       <c r="M3">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -5203,7 +5203,7 @@
         <v>91</v>
       </c>
       <c r="M5">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5326,7 +5326,7 @@
         <v>286</v>
       </c>
       <c r="M8">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5367,7 +5367,7 @@
         <v>79</v>
       </c>
       <c r="M9">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -5408,7 +5408,7 @@
         <v>748</v>
       </c>
       <c r="M10">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5449,7 +5449,7 @@
         <v>1503</v>
       </c>
       <c r="M11">
-        <v>1200</v>
+        <v>1206</v>
       </c>
     </row>
   </sheetData>
@@ -5679,7 +5679,7 @@
         <v>76</v>
       </c>
       <c r="M5">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -5799,7 +5799,7 @@
         <v>436</v>
       </c>
       <c r="M8">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -5881,7 +5881,7 @@
         <v>637</v>
       </c>
       <c r="M10">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -5922,7 +5922,7 @@
         <v>1423</v>
       </c>
       <c r="M11">
-        <v>1151</v>
+        <v>1156</v>
       </c>
     </row>
   </sheetData>
@@ -6269,7 +6269,7 @@
         <v>208</v>
       </c>
       <c r="M8">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6351,7 +6351,7 @@
         <v>2706</v>
       </c>
       <c r="M10">
-        <v>1904</v>
+        <v>1921</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6392,7 +6392,7 @@
         <v>3347</v>
       </c>
       <c r="M11">
-        <v>2412</v>
+        <v>2431</v>
       </c>
     </row>
   </sheetData>
@@ -6499,7 +6499,7 @@
         <v>924</v>
       </c>
       <c r="M2">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -6581,7 +6581,7 @@
         <v>597</v>
       </c>
       <c r="M4">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -6663,7 +6663,7 @@
         <v>782</v>
       </c>
       <c r="M6">
-        <v>576</v>
+        <v>577</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -6704,7 +6704,7 @@
         <v>2405</v>
       </c>
       <c r="M7">
-        <v>1737</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -6745,7 +6745,7 @@
         <v>4416</v>
       </c>
       <c r="M8">
-        <v>3317</v>
+        <v>3333</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -6786,7 +6786,7 @@
         <v>441</v>
       </c>
       <c r="M9">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6827,7 +6827,7 @@
         <v>1149</v>
       </c>
       <c r="M10">
-        <v>903</v>
+        <v>906</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -6868,7 +6868,7 @@
         <v>1778</v>
       </c>
       <c r="M11">
-        <v>1444</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -6950,7 +6950,7 @@
         <v>267</v>
       </c>
       <c r="M13">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -6991,7 +6991,7 @@
         <v>727</v>
       </c>
       <c r="M14">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -7032,7 +7032,7 @@
         <v>808</v>
       </c>
       <c r="M15">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -7155,7 +7155,7 @@
         <v>643</v>
       </c>
       <c r="M18">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -7196,7 +7196,7 @@
         <v>2324</v>
       </c>
       <c r="M19">
-        <v>1597</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -7237,7 +7237,7 @@
         <v>1694</v>
       </c>
       <c r="M20">
-        <v>1289</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -7278,7 +7278,7 @@
         <v>275</v>
       </c>
       <c r="M21">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -7319,7 +7319,7 @@
         <v>383</v>
       </c>
       <c r="M22">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -7401,7 +7401,7 @@
         <v>531</v>
       </c>
       <c r="M24">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -7483,7 +7483,7 @@
         <v>234</v>
       </c>
       <c r="M26">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -7524,7 +7524,7 @@
         <v>1238</v>
       </c>
       <c r="M27">
-        <v>877</v>
+        <v>880</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -7606,7 +7606,7 @@
         <v>3353</v>
       </c>
       <c r="M29">
-        <v>2509</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -7688,7 +7688,7 @@
         <v>1011</v>
       </c>
       <c r="M31">
-        <v>932</v>
+        <v>936</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -7770,7 +7770,7 @@
         <v>2438</v>
       </c>
       <c r="M33">
-        <v>1992</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -7811,7 +7811,7 @@
         <v>701</v>
       </c>
       <c r="M34">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -7852,7 +7852,7 @@
         <v>323</v>
       </c>
       <c r="M35">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7893,7 +7893,7 @@
         <v>1423</v>
       </c>
       <c r="M36">
-        <v>1151</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -7934,7 +7934,7 @@
         <v>2326</v>
       </c>
       <c r="M37">
-        <v>1783</v>
+        <v>1791</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -8057,7 +8057,7 @@
         <v>329</v>
       </c>
       <c r="M40">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -8139,7 +8139,7 @@
         <v>2489</v>
       </c>
       <c r="M42">
-        <v>2398</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -8180,7 +8180,7 @@
         <v>1461</v>
       </c>
       <c r="M43">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -8221,7 +8221,7 @@
         <v>973</v>
       </c>
       <c r="M44">
-        <v>751</v>
+        <v>756</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -8303,7 +8303,7 @@
         <v>300</v>
       </c>
       <c r="M46">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -8344,7 +8344,7 @@
         <v>940</v>
       </c>
       <c r="M47">
-        <v>742</v>
+        <v>745</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -8385,7 +8385,7 @@
         <v>2758</v>
       </c>
       <c r="M48">
-        <v>2081</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -8426,7 +8426,7 @@
         <v>1776</v>
       </c>
       <c r="M49">
-        <v>1394</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -8467,7 +8467,7 @@
         <v>1014</v>
       </c>
       <c r="M50">
-        <v>797</v>
+        <v>801</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -8508,7 +8508,7 @@
         <v>1444</v>
       </c>
       <c r="M51">
-        <v>1158</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -8549,7 +8549,7 @@
         <v>1407</v>
       </c>
       <c r="M52">
-        <v>1025</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -8590,7 +8590,7 @@
         <v>1749</v>
       </c>
       <c r="M53">
-        <v>1426</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -8631,7 +8631,7 @@
         <v>3820</v>
       </c>
       <c r="M54">
-        <v>2804</v>
+        <v>2819</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -8672,7 +8672,7 @@
         <v>1077</v>
       </c>
       <c r="M55">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -8713,7 +8713,7 @@
         <v>619</v>
       </c>
       <c r="M56">
-        <v>384</v>
+        <v>391</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -8754,7 +8754,7 @@
         <v>466</v>
       </c>
       <c r="M57">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -8795,7 +8795,7 @@
         <v>143</v>
       </c>
       <c r="M58">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -8836,7 +8836,7 @@
         <v>297</v>
       </c>
       <c r="M59">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -9000,7 +9000,7 @@
         <v>1382</v>
       </c>
       <c r="M63">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="64" spans="1:13">
@@ -9041,7 +9041,7 @@
         <v>947</v>
       </c>
       <c r="M64">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="65" spans="1:13">
@@ -9082,7 +9082,7 @@
         <v>1383</v>
       </c>
       <c r="M65">
-        <v>1091</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="66" spans="1:13">
@@ -9123,7 +9123,7 @@
         <v>602</v>
       </c>
       <c r="M66">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="67" spans="1:13">
@@ -9164,7 +9164,7 @@
         <v>1914</v>
       </c>
       <c r="M67">
-        <v>1518</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="68" spans="1:13">
@@ -9205,7 +9205,7 @@
         <v>500</v>
       </c>
       <c r="M68">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="69" spans="1:13">
@@ -9246,7 +9246,7 @@
         <v>472</v>
       </c>
       <c r="M69">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="70" spans="1:13">
@@ -9287,7 +9287,7 @@
         <v>651</v>
       </c>
       <c r="M70">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="71" spans="1:13">
@@ -9328,7 +9328,7 @@
         <v>346</v>
       </c>
       <c r="M71">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="72" spans="1:13">
@@ -9369,7 +9369,7 @@
         <v>659</v>
       </c>
       <c r="M72">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
     <row r="73" spans="1:13">
@@ -9410,7 +9410,7 @@
         <v>1346</v>
       </c>
       <c r="M73">
-        <v>975</v>
+        <v>980</v>
       </c>
     </row>
     <row r="74" spans="1:13">
@@ -9492,7 +9492,7 @@
         <v>426</v>
       </c>
       <c r="M75">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="76" spans="1:13">
@@ -9533,7 +9533,7 @@
         <v>3347</v>
       </c>
       <c r="M76">
-        <v>2412</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="77" spans="1:13">
@@ -9615,7 +9615,7 @@
         <v>1577</v>
       </c>
       <c r="M78">
-        <v>919</v>
+        <v>921</v>
       </c>
     </row>
     <row r="79" spans="1:13">
@@ -9656,7 +9656,7 @@
         <v>2083</v>
       </c>
       <c r="M79">
-        <v>1402</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="80" spans="1:13">
@@ -9820,7 +9820,7 @@
         <v>1484</v>
       </c>
       <c r="M83">
-        <v>1121</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="84" spans="1:13">
@@ -9861,7 +9861,7 @@
         <v>843</v>
       </c>
       <c r="M84">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="85" spans="1:13">
@@ -9902,7 +9902,7 @@
         <v>3388</v>
       </c>
       <c r="M85">
-        <v>2693</v>
+        <v>2702</v>
       </c>
     </row>
     <row r="86" spans="1:13">
@@ -9943,7 +9943,7 @@
         <v>903</v>
       </c>
       <c r="M86">
-        <v>767</v>
+        <v>768</v>
       </c>
     </row>
     <row r="87" spans="1:13">
@@ -9984,7 +9984,7 @@
         <v>436</v>
       </c>
       <c r="M87">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="88" spans="1:13">
@@ -10025,7 +10025,7 @@
         <v>873</v>
       </c>
       <c r="M88">
-        <v>642</v>
+        <v>643</v>
       </c>
     </row>
     <row r="89" spans="1:13">
@@ -10066,7 +10066,7 @@
         <v>2031</v>
       </c>
       <c r="M89">
-        <v>1647</v>
+        <v>1653</v>
       </c>
     </row>
     <row r="90" spans="1:13">
@@ -10107,7 +10107,7 @@
         <v>1084</v>
       </c>
       <c r="M90">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="91" spans="1:13">
@@ -10148,7 +10148,7 @@
         <v>967</v>
       </c>
       <c r="M91">
-        <v>722</v>
+        <v>727</v>
       </c>
     </row>
     <row r="92" spans="1:13">
@@ -10189,7 +10189,7 @@
         <v>316</v>
       </c>
       <c r="M92">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="93" spans="1:13">
@@ -10230,7 +10230,7 @@
         <v>801</v>
       </c>
       <c r="M93">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
     <row r="94" spans="1:13">
@@ -10271,7 +10271,7 @@
         <v>2666</v>
       </c>
       <c r="M94">
-        <v>2120</v>
+        <v>2123</v>
       </c>
     </row>
     <row r="95" spans="1:13">
@@ -10312,7 +10312,7 @@
         <v>1239</v>
       </c>
       <c r="M95">
-        <v>944</v>
+        <v>949</v>
       </c>
     </row>
     <row r="96" spans="1:13">
@@ -10353,7 +10353,7 @@
         <v>1357</v>
       </c>
       <c r="M96">
-        <v>854</v>
+        <v>859</v>
       </c>
     </row>
     <row r="97" spans="1:13">
@@ -10394,7 +10394,7 @@
         <v>1716</v>
       </c>
       <c r="M97">
-        <v>1157</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="98" spans="1:13">
@@ -10435,7 +10435,7 @@
         <v>1125</v>
       </c>
       <c r="M98">
-        <v>935</v>
+        <v>937</v>
       </c>
     </row>
     <row r="99" spans="1:13">
@@ -10476,7 +10476,7 @@
         <v>1503</v>
       </c>
       <c r="M99">
-        <v>1200</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="100" spans="1:13">
@@ -10558,7 +10558,7 @@
         <v>104496</v>
       </c>
       <c r="M101">
-        <v>78476</v>
+        <v>78780</v>
       </c>
     </row>
   </sheetData>
@@ -10767,7 +10767,7 @@
         <v>36</v>
       </c>
       <c r="M2">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -10887,7 +10887,7 @@
         <v>124</v>
       </c>
       <c r="M5">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -11077,7 +11077,7 @@
         <v>1377</v>
       </c>
       <c r="M10">
-        <v>1047</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -11118,7 +11118,7 @@
         <v>1776</v>
       </c>
       <c r="M11">
-        <v>1394</v>
+        <v>1400</v>
       </c>
     </row>
   </sheetData>
@@ -11447,7 +11447,7 @@
         <v>65</v>
       </c>
       <c r="M8">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -11570,7 +11570,7 @@
         <v>297</v>
       </c>
       <c r="M11">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -11677,7 +11677,7 @@
         <v>59</v>
       </c>
       <c r="M2">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -11996,7 +11996,7 @@
         <v>725</v>
       </c>
       <c r="M10">
-        <v>520</v>
+        <v>521</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12836,7 +12836,7 @@
         <v>448</v>
       </c>
       <c r="M10">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -12877,7 +12877,7 @@
         <v>659</v>
       </c>
       <c r="M11">
-        <v>472</v>
+        <v>475</v>
       </c>
     </row>
   </sheetData>
@@ -13025,7 +13025,7 @@
         <v>234</v>
       </c>
       <c r="M3">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -13107,7 +13107,7 @@
         <v>136</v>
       </c>
       <c r="M5">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13230,7 +13230,7 @@
         <v>497</v>
       </c>
       <c r="M8">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13271,7 +13271,7 @@
         <v>190</v>
       </c>
       <c r="M9">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13312,7 +13312,7 @@
         <v>1164</v>
       </c>
       <c r="M10">
-        <v>1169</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13353,7 +13353,7 @@
         <v>2489</v>
       </c>
       <c r="M11">
-        <v>2398</v>
+        <v>2405</v>
       </c>
     </row>
   </sheetData>
@@ -13501,7 +13501,7 @@
         <v>293</v>
       </c>
       <c r="M3">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -13583,7 +13583,7 @@
         <v>95</v>
       </c>
       <c r="M5">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13747,7 +13747,7 @@
         <v>175</v>
       </c>
       <c r="M9">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13788,7 +13788,7 @@
         <v>739</v>
       </c>
       <c r="M10">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13829,7 +13829,7 @@
         <v>1914</v>
       </c>
       <c r="M11">
-        <v>1518</v>
+        <v>1526</v>
       </c>
     </row>
   </sheetData>
@@ -15074,7 +15074,7 @@
         <v>357</v>
       </c>
       <c r="M8">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -15156,7 +15156,7 @@
         <v>2932</v>
       </c>
       <c r="M10">
-        <v>2150</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15197,7 +15197,7 @@
         <v>3820</v>
       </c>
       <c r="M11">
-        <v>2804</v>
+        <v>2819</v>
       </c>
     </row>
   </sheetData>
@@ -15345,7 +15345,7 @@
         <v>19</v>
       </c>
       <c r="M3">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -15614,7 +15614,7 @@
         <v>408</v>
       </c>
       <c r="M10">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -15655,7 +15655,7 @@
         <v>597</v>
       </c>
       <c r="M11">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -16072,7 +16072,7 @@
         <v>1950</v>
       </c>
       <c r="M10">
-        <v>1525</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16113,7 +16113,7 @@
         <v>2666</v>
       </c>
       <c r="M11">
-        <v>2120</v>
+        <v>2123</v>
       </c>
     </row>
   </sheetData>
@@ -16498,7 +16498,7 @@
         <v>37</v>
       </c>
       <c r="M9">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -16539,7 +16539,7 @@
         <v>597</v>
       </c>
       <c r="M10">
-        <v>493</v>
+        <v>497</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -16580,7 +16580,7 @@
         <v>973</v>
       </c>
       <c r="M11">
-        <v>751</v>
+        <v>756</v>
       </c>
     </row>
   </sheetData>
@@ -16974,7 +16974,7 @@
         <v>82</v>
       </c>
       <c r="M9">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -17015,7 +17015,7 @@
         <v>974</v>
       </c>
       <c r="M10">
-        <v>549</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17056,7 +17056,7 @@
         <v>1577</v>
       </c>
       <c r="M11">
-        <v>919</v>
+        <v>921</v>
       </c>
     </row>
   </sheetData>
@@ -17409,7 +17409,7 @@
         <v>102</v>
       </c>
       <c r="M8">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -17491,7 +17491,7 @@
         <v>168</v>
       </c>
       <c r="M10">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17532,7 +17532,7 @@
         <v>441</v>
       </c>
       <c r="M11">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -17747,7 +17747,7 @@
         <v>66</v>
       </c>
       <c r="M5">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -17940,7 +17940,7 @@
         <v>789</v>
       </c>
       <c r="M10">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -17981,7 +17981,7 @@
         <v>1125</v>
       </c>
       <c r="M11">
-        <v>935</v>
+        <v>937</v>
       </c>
     </row>
   </sheetData>
@@ -18383,7 +18383,7 @@
         <v>179</v>
       </c>
       <c r="M10">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18424,7 +18424,7 @@
         <v>300</v>
       </c>
       <c r="M11">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -18859,7 +18859,7 @@
         <v>730</v>
       </c>
       <c r="M10">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -18900,7 +18900,7 @@
         <v>1694</v>
       </c>
       <c r="M11">
-        <v>1289</v>
+        <v>1291</v>
       </c>
     </row>
   </sheetData>
@@ -19007,7 +19007,7 @@
         <v>249</v>
       </c>
       <c r="M2">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -19130,7 +19130,7 @@
         <v>171</v>
       </c>
       <c r="M5">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -19171,7 +19171,7 @@
         <v>52</v>
       </c>
       <c r="M6">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -19253,7 +19253,7 @@
         <v>417</v>
       </c>
       <c r="M8">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -19294,7 +19294,7 @@
         <v>209</v>
       </c>
       <c r="M9">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -19335,7 +19335,7 @@
         <v>895</v>
       </c>
       <c r="M10">
-        <v>680</v>
+        <v>683</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19376,7 +19376,7 @@
         <v>2326</v>
       </c>
       <c r="M11">
-        <v>1783</v>
+        <v>1791</v>
       </c>
     </row>
   </sheetData>
@@ -19524,7 +19524,7 @@
         <v>141</v>
       </c>
       <c r="M3">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -19811,7 +19811,7 @@
         <v>679</v>
       </c>
       <c r="M10">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -19852,7 +19852,7 @@
         <v>1407</v>
       </c>
       <c r="M11">
-        <v>1025</v>
+        <v>1029</v>
       </c>
     </row>
   </sheetData>
@@ -19959,7 +19959,7 @@
         <v>105</v>
       </c>
       <c r="M2">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -20205,7 +20205,7 @@
         <v>284</v>
       </c>
       <c r="M8">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -20287,7 +20287,7 @@
         <v>491</v>
       </c>
       <c r="M10">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20328,7 +20328,7 @@
         <v>1239</v>
       </c>
       <c r="M11">
-        <v>944</v>
+        <v>949</v>
       </c>
     </row>
   </sheetData>
@@ -20763,7 +20763,7 @@
         <v>433</v>
       </c>
       <c r="M10">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -20804,7 +20804,7 @@
         <v>873</v>
       </c>
       <c r="M11">
-        <v>642</v>
+        <v>643</v>
       </c>
     </row>
   </sheetData>
@@ -21133,7 +21133,7 @@
         <v>119</v>
       </c>
       <c r="M8">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21215,7 +21215,7 @@
         <v>161</v>
       </c>
       <c r="M10">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -21256,7 +21256,7 @@
         <v>346</v>
       </c>
       <c r="M11">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -21404,7 +21404,7 @@
         <v>137</v>
       </c>
       <c r="M3">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -21609,7 +21609,7 @@
         <v>233</v>
       </c>
       <c r="M8">
-        <v>184</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -21650,7 +21650,7 @@
         <v>104</v>
       </c>
       <c r="M9">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -21732,7 +21732,7 @@
         <v>1383</v>
       </c>
       <c r="M11">
-        <v>1091</v>
+        <v>1096</v>
       </c>
     </row>
   </sheetData>
@@ -22073,7 +22073,7 @@
         <v>56</v>
       </c>
       <c r="M8">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22196,7 +22196,7 @@
         <v>466</v>
       </c>
       <c r="M11">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
   </sheetData>
@@ -22549,7 +22549,7 @@
         <v>250</v>
       </c>
       <c r="M8">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -22631,7 +22631,7 @@
         <v>379</v>
       </c>
       <c r="M10">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -22672,7 +22672,7 @@
         <v>967</v>
       </c>
       <c r="M11">
-        <v>722</v>
+        <v>727</v>
       </c>
     </row>
   </sheetData>
@@ -22922,7 +22922,7 @@
         <v>2</v>
       </c>
       <c r="M6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -22977,7 +22977,7 @@
         <v>82</v>
       </c>
       <c r="M8">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23100,7 +23100,7 @@
         <v>651</v>
       </c>
       <c r="M11">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -23248,7 +23248,7 @@
         <v>57</v>
       </c>
       <c r="M3">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -23312,7 +23312,7 @@
         <v>70</v>
       </c>
       <c r="M5">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -23423,7 +23423,7 @@
         <v>189</v>
       </c>
       <c r="M8">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23546,7 +23546,7 @@
         <v>1461</v>
       </c>
       <c r="M11">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -23653,7 +23653,7 @@
         <v>185</v>
       </c>
       <c r="M2">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -23694,7 +23694,7 @@
         <v>195</v>
       </c>
       <c r="M3">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -23776,7 +23776,7 @@
         <v>149</v>
       </c>
       <c r="M5">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -23899,7 +23899,7 @@
         <v>468</v>
       </c>
       <c r="M8">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -23940,7 +23940,7 @@
         <v>161</v>
       </c>
       <c r="M9">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -23981,7 +23981,7 @@
         <v>860</v>
       </c>
       <c r="M10">
-        <v>590</v>
+        <v>594</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24022,7 +24022,7 @@
         <v>2083</v>
       </c>
       <c r="M11">
-        <v>1402</v>
+        <v>1411</v>
       </c>
     </row>
   </sheetData>
@@ -24339,7 +24339,7 @@
         <v>85</v>
       </c>
       <c r="M8">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -24462,7 +24462,7 @@
         <v>602</v>
       </c>
       <c r="M11">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
   </sheetData>
@@ -24870,7 +24870,7 @@
         <v>301</v>
       </c>
       <c r="M10">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -24911,7 +24911,7 @@
         <v>436</v>
       </c>
       <c r="M11">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>
@@ -25018,7 +25018,7 @@
         <v>34</v>
       </c>
       <c r="M2">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -25331,7 +25331,7 @@
         <v>747</v>
       </c>
       <c r="M10">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25372,7 +25372,7 @@
         <v>1014</v>
       </c>
       <c r="M11">
-        <v>797</v>
+        <v>801</v>
       </c>
     </row>
   </sheetData>
@@ -25602,7 +25602,7 @@
         <v>223</v>
       </c>
       <c r="M5">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -25725,7 +25725,7 @@
         <v>637</v>
       </c>
       <c r="M8">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -25766,7 +25766,7 @@
         <v>286</v>
       </c>
       <c r="M9">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -25807,7 +25807,7 @@
         <v>1267</v>
       </c>
       <c r="M10">
-        <v>961</v>
+        <v>965</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -25848,7 +25848,7 @@
         <v>3353</v>
       </c>
       <c r="M11">
-        <v>2509</v>
+        <v>2518</v>
       </c>
     </row>
   </sheetData>
@@ -26262,7 +26262,7 @@
         <v>189</v>
       </c>
       <c r="M10">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26303,7 +26303,7 @@
         <v>383</v>
       </c>
       <c r="M11">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>
@@ -26565,7 +26565,7 @@
         <v>16</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -26723,7 +26723,7 @@
         <v>544</v>
       </c>
       <c r="M10">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -26764,7 +26764,7 @@
         <v>947</v>
       </c>
       <c r="M11">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
   </sheetData>
@@ -27090,7 +27090,7 @@
         <v>57</v>
       </c>
       <c r="M8">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -27172,7 +27172,7 @@
         <v>338</v>
       </c>
       <c r="M10">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27213,7 +27213,7 @@
         <v>472</v>
       </c>
       <c r="M11">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
   </sheetData>
@@ -27443,7 +27443,7 @@
         <v>136</v>
       </c>
       <c r="M5">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -27645,7 +27645,7 @@
         <v>1423</v>
       </c>
       <c r="M10">
-        <v>1204</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -27686,7 +27686,7 @@
         <v>2031</v>
       </c>
       <c r="M11">
-        <v>1647</v>
+        <v>1653</v>
       </c>
     </row>
   </sheetData>
@@ -28121,7 +28121,7 @@
         <v>585</v>
       </c>
       <c r="M10">
-        <v>530</v>
+        <v>531</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28162,7 +28162,7 @@
         <v>1077</v>
       </c>
       <c r="M11">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
   </sheetData>
@@ -28474,7 +28474,7 @@
         <v>9</v>
       </c>
       <c r="M7">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -28556,7 +28556,7 @@
         <v>164</v>
       </c>
       <c r="M9">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -28597,7 +28597,7 @@
         <v>1121</v>
       </c>
       <c r="M10">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -28638,7 +28638,7 @@
         <v>2324</v>
       </c>
       <c r="M11">
-        <v>1597</v>
+        <v>1602</v>
       </c>
     </row>
   </sheetData>
@@ -28991,7 +28991,7 @@
         <v>122</v>
       </c>
       <c r="M8">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -29032,7 +29032,7 @@
         <v>37</v>
       </c>
       <c r="M9">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -29114,7 +29114,7 @@
         <v>808</v>
       </c>
       <c r="M11">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
   </sheetData>
@@ -29467,7 +29467,7 @@
         <v>377</v>
       </c>
       <c r="M8">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -29549,7 +29549,7 @@
         <v>491</v>
       </c>
       <c r="M10">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -29590,7 +29590,7 @@
         <v>1484</v>
       </c>
       <c r="M11">
-        <v>1121</v>
+        <v>1124</v>
       </c>
     </row>
   </sheetData>
@@ -30164,7 +30164,7 @@
         <v>132</v>
       </c>
       <c r="M2">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -30368,6 +30368,9 @@
       <c r="L7">
         <v>4</v>
       </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
@@ -30407,7 +30410,7 @@
         <v>285</v>
       </c>
       <c r="M8">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -30489,7 +30492,7 @@
         <v>1041</v>
       </c>
       <c r="M10">
-        <v>872</v>
+        <v>876</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30530,7 +30533,7 @@
         <v>1778</v>
       </c>
       <c r="M11">
-        <v>1444</v>
+        <v>1451</v>
       </c>
     </row>
   </sheetData>
@@ -30908,7 +30911,7 @@
         <v>582</v>
       </c>
       <c r="M10">
-        <v>356</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -30949,7 +30952,7 @@
         <v>619</v>
       </c>
       <c r="M11">
-        <v>384</v>
+        <v>391</v>
       </c>
     </row>
   </sheetData>
@@ -31378,7 +31381,7 @@
         <v>1104</v>
       </c>
       <c r="M10">
-        <v>735</v>
+        <v>736</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31419,7 +31422,7 @@
         <v>1716</v>
       </c>
       <c r="M11">
-        <v>1157</v>
+        <v>1158</v>
       </c>
     </row>
   </sheetData>
@@ -31646,7 +31649,7 @@
         <v>40</v>
       </c>
       <c r="M5">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -31836,7 +31839,7 @@
         <v>306</v>
       </c>
       <c r="M10">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -31877,7 +31880,7 @@
         <v>531</v>
       </c>
       <c r="M11">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -32104,7 +32107,7 @@
         <v>41</v>
       </c>
       <c r="M5">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -32309,7 +32312,7 @@
         <v>446</v>
       </c>
       <c r="M10">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32498,7 +32501,7 @@
         <v>51</v>
       </c>
       <c r="M3">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -32785,7 +32788,7 @@
         <v>266</v>
       </c>
       <c r="M10">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -32826,7 +32829,7 @@
         <v>643</v>
       </c>
       <c r="M11">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -32974,7 +32977,7 @@
         <v>68</v>
       </c>
       <c r="M3">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -33261,7 +33264,7 @@
         <v>478</v>
       </c>
       <c r="M10">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33302,7 +33305,7 @@
         <v>1084</v>
       </c>
       <c r="M11">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
   </sheetData>
@@ -33643,7 +33646,7 @@
         <v>192</v>
       </c>
       <c r="M8">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -33725,7 +33728,7 @@
         <v>553</v>
       </c>
       <c r="M10">
-        <v>422</v>
+        <v>424</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -33766,7 +33769,7 @@
         <v>940</v>
       </c>
       <c r="M11">
-        <v>742</v>
+        <v>745</v>
       </c>
     </row>
   </sheetData>
@@ -34080,7 +34083,7 @@
         <v>103</v>
       </c>
       <c r="M8">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34162,7 +34165,7 @@
         <v>152</v>
       </c>
       <c r="M10">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34203,7 +34206,7 @@
         <v>329</v>
       </c>
       <c r="M11">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -34553,7 +34556,7 @@
         <v>308</v>
       </c>
       <c r="M8">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -34635,7 +34638,7 @@
         <v>813</v>
       </c>
       <c r="M10">
-        <v>705</v>
+        <v>706</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -34676,7 +34679,7 @@
         <v>1444</v>
       </c>
       <c r="M11">
-        <v>1158</v>
+        <v>1160</v>
       </c>
     </row>
   </sheetData>
@@ -34783,7 +34786,7 @@
         <v>70</v>
       </c>
       <c r="M2">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -35111,7 +35114,7 @@
         <v>400</v>
       </c>
       <c r="M10">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35152,7 +35155,7 @@
         <v>843</v>
       </c>
       <c r="M11">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
   </sheetData>
@@ -35505,7 +35508,7 @@
         <v>206</v>
       </c>
       <c r="M8">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -35546,7 +35549,7 @@
         <v>40</v>
       </c>
       <c r="M9">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -35587,7 +35590,7 @@
         <v>896</v>
       </c>
       <c r="M10">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -35628,7 +35631,7 @@
         <v>1346</v>
       </c>
       <c r="M11">
-        <v>975</v>
+        <v>980</v>
       </c>
     </row>
   </sheetData>
@@ -35735,7 +35738,7 @@
         <v>78</v>
       </c>
       <c r="M2">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -35776,7 +35779,7 @@
         <v>68</v>
       </c>
       <c r="M3">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -35858,7 +35861,7 @@
         <v>104</v>
       </c>
       <c r="M5">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -36063,7 +36066,7 @@
         <v>761</v>
       </c>
       <c r="M10">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36104,7 +36107,7 @@
         <v>1357</v>
       </c>
       <c r="M11">
-        <v>854</v>
+        <v>859</v>
       </c>
     </row>
   </sheetData>
@@ -36445,7 +36448,7 @@
         <v>125</v>
       </c>
       <c r="M8">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -36527,7 +36530,7 @@
         <v>812</v>
       </c>
       <c r="M10">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36568,7 +36571,7 @@
         <v>1238</v>
       </c>
       <c r="M11">
-        <v>877</v>
+        <v>880</v>
       </c>
     </row>
   </sheetData>
@@ -36943,7 +36946,7 @@
         <v>204</v>
       </c>
       <c r="M10">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -36984,7 +36987,7 @@
         <v>267</v>
       </c>
       <c r="M11">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -38037,7 +38040,7 @@
         <v>19</v>
       </c>
       <c r="M5">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -38130,7 +38133,7 @@
         <v>33</v>
       </c>
       <c r="M8">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -38253,7 +38256,7 @@
         <v>234</v>
       </c>
       <c r="M11">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -38676,7 +38679,7 @@
         <v>151</v>
       </c>
       <c r="M10">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -38717,7 +38720,7 @@
         <v>316</v>
       </c>
       <c r="M11">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -38824,7 +38827,7 @@
         <v>62</v>
       </c>
       <c r="M2">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -38947,7 +38950,7 @@
         <v>42</v>
       </c>
       <c r="M5">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -39152,7 +39155,7 @@
         <v>532</v>
       </c>
       <c r="M10">
-        <v>399</v>
+        <v>403</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39193,7 +39196,7 @@
         <v>924</v>
       </c>
       <c r="M11">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
   </sheetData>
@@ -39601,7 +39604,7 @@
         <v>328</v>
       </c>
       <c r="M10">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -39642,7 +39645,7 @@
         <v>500</v>
       </c>
       <c r="M11">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -40023,7 +40026,7 @@
         <v>166</v>
       </c>
       <c r="M10">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40064,7 +40067,7 @@
         <v>275</v>
       </c>
       <c r="M11">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -40839,7 +40842,7 @@
         <v>250</v>
       </c>
       <c r="M8">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -40921,7 +40924,7 @@
         <v>2025</v>
       </c>
       <c r="M10">
-        <v>1615</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -40962,7 +40965,7 @@
         <v>2758</v>
       </c>
       <c r="M11">
-        <v>2081</v>
+        <v>2085</v>
       </c>
     </row>
   </sheetData>
@@ -41831,7 +41834,7 @@
         <v>661</v>
       </c>
       <c r="M10">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -41872,7 +41875,7 @@
         <v>903</v>
       </c>
       <c r="M11">
-        <v>767</v>
+        <v>768</v>
       </c>
     </row>
   </sheetData>
@@ -42295,7 +42298,7 @@
         <v>426</v>
       </c>
       <c r="M10">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -42336,7 +42339,7 @@
         <v>727</v>
       </c>
       <c r="M11">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
   </sheetData>
@@ -43074,7 +43077,7 @@
         <v>9</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -43270,7 +43273,7 @@
         <v>426</v>
       </c>
       <c r="M11">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -44088,7 +44091,7 @@
         <v>265</v>
       </c>
       <c r="M10">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -44129,7 +44132,7 @@
         <v>323</v>
       </c>
       <c r="M11">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -44277,7 +44280,7 @@
         <v>32</v>
       </c>
       <c r="M3">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -44602,7 +44605,7 @@
         <v>701</v>
       </c>
       <c r="M11">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
   </sheetData>
@@ -45131,7 +45134,7 @@
         <v>38</v>
       </c>
       <c r="M2">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -45172,7 +45175,7 @@
         <v>31</v>
       </c>
       <c r="M3">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -45365,7 +45368,7 @@
         <v>155</v>
       </c>
       <c r="M8">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -45447,7 +45450,7 @@
         <v>485</v>
       </c>
       <c r="M10">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45488,7 +45491,7 @@
         <v>801</v>
       </c>
       <c r="M11">
-        <v>588</v>
+        <v>593</v>
       </c>
     </row>
   </sheetData>
@@ -45595,7 +45598,7 @@
         <v>265</v>
       </c>
       <c r="M2">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -45636,7 +45639,7 @@
         <v>341</v>
       </c>
       <c r="M3">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -45882,7 +45885,7 @@
         <v>271</v>
       </c>
       <c r="M9">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -45923,7 +45926,7 @@
         <v>873</v>
       </c>
       <c r="M10">
-        <v>756</v>
+        <v>762</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -45964,7 +45967,7 @@
         <v>2438</v>
       </c>
       <c r="M11">
-        <v>1992</v>
+        <v>2002</v>
       </c>
     </row>
   </sheetData>
@@ -46306,7 +46309,7 @@
         <v>129</v>
       </c>
       <c r="M10">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -46347,7 +46350,7 @@
         <v>143</v>
       </c>
       <c r="M11">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -47044,7 +47047,7 @@
         <v>18</v>
       </c>
       <c r="M8">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -47126,7 +47129,7 @@
         <v>200</v>
       </c>
       <c r="M10">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:13">

</xml_diff>